<commit_message>
Use the Drake Client Contact List as the client list template
- Reads the Individual Clients tab and skips the template's example row
- Converts Drake's capitalised names (JANE -> Jane, O'BRIEN -> O'Brien)
- Sends to the spouse email when there is no taxpayer email
- Adds a Client Type column to the template and a --new option
- Skips duplicate emails within one run

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019sSAMAxBZX69MhEJJ74rUi
</commit_message>
<xml_diff>
--- a/tax_doc_requests/sample_clients.xlsx
+++ b/tax_doc_requests/sample_clients.xlsx
@@ -7,17 +7,28 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clients" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Individual Clients" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Business Clients" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings &amp; Drake Status" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Still Missing" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Individual Clients'!$A$1:$N$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Business Clients'!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Findings &amp; Drake Status'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Still Missing'!$A$1:$B$1</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
+  </numFmts>
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,18 +37,60 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Arial"/>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00808080"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007F6000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00375623"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE699"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8CBAD"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,13 +98,46 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,164 +503,579 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="37" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="23" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="32" customWidth="1" min="12" max="12"/>
+    <col width="90" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Taxpayer First Name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Taxpayer Last Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Taxpayer Date of Birth</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Taxpayer Contact Number</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Taxpayer Other Phone</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Taxpayer Email</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Spouse First Name</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Spouse Last Name</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Spouse Date of Birth</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Spouse Contact Number</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Spouse Other Phone</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Spouse Email</t>
+        </is>
+      </c>
+      <c r="M1" s="6" t="inlineStr">
+        <is>
+          <t>Found in Outlook - source / notes</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Client Type (New / Returning)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>JANE</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t>SAMPLE</t>
+        </is>
+      </c>
+      <c r="C2" s="16" t="n">
+        <v>29221</v>
+      </c>
+      <c r="D2" s="15" t="inlineStr">
+        <is>
+          <t>(555) 010-0001</t>
+        </is>
+      </c>
+      <c r="E2" s="15" t="inlineStr"/>
+      <c r="F2" s="15" t="inlineStr">
+        <is>
+          <t>jane.sample@example.com</t>
+        </is>
+      </c>
+      <c r="G2" s="15" t="inlineStr">
+        <is>
+          <t>JOHN</t>
+        </is>
+      </c>
+      <c r="H2" s="15" t="inlineStr">
+        <is>
+          <t>SAMPLE</t>
+        </is>
+      </c>
+      <c r="I2" s="16" t="n">
+        <v>29619</v>
+      </c>
+      <c r="J2" s="15" t="inlineStr"/>
+      <c r="K2" s="15" t="inlineStr"/>
+      <c r="L2" s="17" t="inlineStr">
+        <is>
+          <t>john.sample@example.com</t>
+        </is>
+      </c>
+      <c r="M2" s="15" t="inlineStr">
+        <is>
+          <t>Spouse email: EXAMPLE ROW - delete. Source of any value found outside Drake goes here</t>
+        </is>
+      </c>
+      <c r="N2" s="15" t="inlineStr">
+        <is>
+          <t>Returning</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>ALEX</t>
+        </is>
+      </c>
+      <c r="B3" s="15" t="inlineStr">
+        <is>
+          <t>EXAMPLE</t>
+        </is>
+      </c>
+      <c r="C3" s="16" t="n">
+        <v>32935</v>
+      </c>
+      <c r="D3" s="15" t="inlineStr">
+        <is>
+          <t>(555) 010-0003</t>
+        </is>
+      </c>
+      <c r="E3" s="15" t="n"/>
+      <c r="F3" s="15" t="inlineStr">
+        <is>
+          <t>alex@example.com</t>
+        </is>
+      </c>
+      <c r="G3" s="15" t="n"/>
+      <c r="H3" s="15" t="n"/>
+      <c r="I3" s="16" t="n"/>
+      <c r="J3" s="15" t="n"/>
+      <c r="K3" s="15" t="n"/>
+      <c r="L3" s="15" t="n"/>
+      <c r="M3" s="15" t="n"/>
+      <c r="N3" s="15" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>PRIYA</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>DEMO</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="n">
+        <v>31141</v>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>(555) 010-0004</t>
+        </is>
+      </c>
+      <c r="E4" s="15" t="n"/>
+      <c r="F4" s="15" t="inlineStr">
+        <is>
+          <t>priya.demo@example.com</t>
+        </is>
+      </c>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>RAVI</t>
+        </is>
+      </c>
+      <c r="H4" s="15" t="inlineStr">
+        <is>
+          <t>TEST</t>
+        </is>
+      </c>
+      <c r="I4" s="16" t="n">
+        <v>30807</v>
+      </c>
+      <c r="J4" s="15" t="n"/>
+      <c r="K4" s="15" t="n"/>
+      <c r="L4" s="15" t="inlineStr">
+        <is>
+          <t>ravi.test@example.com</t>
+        </is>
+      </c>
+      <c r="M4" s="15" t="n"/>
+      <c r="N4" s="15" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>MARY</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>O'BRIEN</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="n">
+        <v>25725</v>
+      </c>
+      <c r="D5" s="15" t="inlineStr">
+        <is>
+          <t>(555) 010-0005</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="n"/>
+      <c r="F5" s="15" t="n"/>
+      <c r="G5" s="15" t="inlineStr">
+        <is>
+          <t>PAT</t>
+        </is>
+      </c>
+      <c r="H5" s="15" t="inlineStr">
+        <is>
+          <t>O'BRIEN</t>
+        </is>
+      </c>
+      <c r="I5" s="16" t="n">
+        <v>26121</v>
+      </c>
+      <c r="J5" s="15" t="n"/>
+      <c r="K5" s="15" t="n"/>
+      <c r="L5" s="15" t="inlineStr">
+        <is>
+          <t>pat.obrien@example.com</t>
+        </is>
+      </c>
+      <c r="M5" s="15" t="n"/>
+      <c r="N5" s="15" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:N5"/>
+  <dataValidations count="1">
+    <dataValidation sqref="N2:N5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Client Type" prompt="New or Returning. Blank = Returning." type="list">
+      <formula1>"New,Returning"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="37" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="31" customWidth="1" min="4" max="4"/>
+    <col width="90" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Business Name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Contact Number</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Other Phone</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Found in Outlook - source / notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>EXAMPLE HOLDINGS LLC</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t>(555) 010-0002</t>
+        </is>
+      </c>
+      <c r="C2" s="15" t="inlineStr"/>
+      <c r="D2" s="17" t="inlineStr">
+        <is>
+          <t>owner@example.com</t>
+        </is>
+      </c>
+      <c r="E2" s="15" t="inlineStr">
+        <is>
+          <t>Email: EXAMPLE ROW - delete</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="95" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="58" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>First Name</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Last Name</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Spouse First Name</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Spouse Last Name</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Spouse Email</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Filing Status</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Client Type</t>
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>Value added</t>
+        </is>
+      </c>
+      <c r="D1" s="11" t="inlineStr">
+        <is>
+          <t>Where it came from</t>
+        </is>
+      </c>
+      <c r="E1" s="11" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F1" s="11" t="inlineStr">
+        <is>
+          <t>Entered in Drake?</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Jane</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Sample</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>John</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>jane.sample@example.com</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>Jane Sample</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t>Spouse email</t>
+        </is>
+      </c>
+      <c r="C2" s="15" t="inlineStr">
         <is>
           <t>john.sample@example.com</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>MFJ</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Returning</t>
+      <c r="D2" s="15" t="inlineStr">
+        <is>
+          <t>HelloSign e-file authorization signed MM/DD/YYYY</t>
+        </is>
+      </c>
+      <c r="E2" s="15" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="F2" s="15" t="inlineStr">
+        <is>
+          <t>Yes - verified MM/DD/YYYY</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="B1" s="12" t="inlineStr">
+        <is>
+          <t>Still missing</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>JANE SAMPLE</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t>Spouse phone (JOHN)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="130" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>TEMPLATE - Drake client contact list (no client data). Row 2 on each tab is a fictional example; delete it before use.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>Source data: Drake Tax Report Manager &gt; My Reports &gt; custom "Client Contact List" (tax return data, all return types), exported to CSV. CSV has 2 title rows, then headers, and a final "Totals (N)" row to drop.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Alex</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Example</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>alex@example.com</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Single</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>New</t>
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>Report columns: Taxpayer Name, Taxpayer First/Last Name, Taxpayer Date of Birth, Taxpayer Cell/Daytime/Evening Phone, Taxpayer Email Address, Spouse First/Last Name, Spouse Email Address, Spouse Evening/Cell Phone, Spouse Date of Birth, Spouse Daytime Phone, Phone Number, Email Address.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Priya</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Demo</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Ravi</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>priya.demo@example.com</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>MFJ</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>New</t>
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Individual vs business: rows with a blank Taxpayer First Name are entities and go to Business Clients.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>De-duplication: Drake repeats a joint return once per email; group on every column except the generic Phone Number / Email Address and keep one row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Contact Number = cell, else daytime, else evening (then generic Phone Number); any further distinct number goes in Other Phone. Phones formatted (XXX) XXX-XXXX; emails lower-case.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Colour key: green fill = value found outside Drake and backed by a specific email; amber fill = likely match, needs confirmation. Source of each added value goes in the last column and on Findings &amp; Drake Status.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Still Missing lists every blank taxpayer phone/email, spouse phone/email (only when a spouse exists), and business phone/email.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>Font: Arial 10, header row bold white on navy (spouse columns on dark gold, Outlook/notes columns on dark green), frozen panes, autofilter on header row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Client Type (column N, added for the tax document request script): New or Returning. Blank = Returning. New clients are asked for last year's return and Driver's License(s); both spouses when there is a spouse.</t>
         </is>
       </c>
     </row>

</xml_diff>